<commit_message>
Changed some opacity and other stuff
</commit_message>
<xml_diff>
--- a/speedway-data.xlsx
+++ b/speedway-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliver/Downloads/SPX_1_3_0_macos64/ASSETS/templates/Speedway GFX/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E74600C2-AF11-394F-A5DC-73217B534559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5710865-BC69-174F-AB2D-19AD98F3BF95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="28800" windowHeight="17500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Event Info" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="47">
   <si>
     <t>Event Information</t>
   </si>
@@ -142,55 +142,40 @@
     <t>Mercury Baypark</t>
   </si>
   <si>
-    <t>Midget Champs</t>
-  </si>
-  <si>
     <t>#BayparkSpeedway</t>
   </si>
   <si>
     <t>Laps</t>
   </si>
   <si>
-    <t>Heat 10</t>
-  </si>
-  <si>
-    <t>Heat 1 1</t>
-  </si>
-  <si>
-    <t>Heat 12</t>
-  </si>
-  <si>
     <t>Sprintcar</t>
   </si>
   <si>
-    <t>Six Shooter</t>
-  </si>
-  <si>
     <t>Heat 4</t>
   </si>
   <si>
-    <t>Heat 13</t>
-  </si>
-  <si>
-    <t>Heat 14</t>
-  </si>
-  <si>
-    <t>Heat 15</t>
-  </si>
-  <si>
-    <t>Heat 5</t>
-  </si>
-  <si>
-    <t>Semi Main</t>
-  </si>
-  <si>
-    <t>Midget</t>
-  </si>
-  <si>
     <t>Heat</t>
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>Supersaloon</t>
+  </si>
+  <si>
+    <t>Race 1</t>
+  </si>
+  <si>
+    <t>Heat 3</t>
+  </si>
+  <si>
+    <t>Race 2</t>
+  </si>
+  <si>
+    <t>Pole Shuffle - Top 6</t>
+  </si>
+  <si>
+    <t>Race 3</t>
   </si>
 </sst>
 </file>
@@ -634,11 +619,8 @@
       <c r="A3" t="s">
         <v>34</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>35</v>
-      </c>
-      <c r="C3" t="s">
-        <v>36</v>
       </c>
       <c r="D3" t="s">
         <v>17</v>
@@ -802,10 +784,10 @@
         <v>12</v>
       </c>
       <c r="C1" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="D1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E1" t="s">
         <v>22</v>
@@ -818,11 +800,8 @@
       <c r="A2" s="2">
         <v>0.38194444444444442</v>
       </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
       <c r="C2" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="D2">
         <v>6</v>
@@ -839,16 +818,16 @@
         <v>0.3888888888888889</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="D3">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="F3" t="b">
         <v>0</v>
@@ -859,16 +838,16 @@
         <v>0.39583333333333298</v>
       </c>
       <c r="B4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="D4">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="F4" t="b">
         <v>0</v>
@@ -879,16 +858,16 @@
         <v>0.40277777777777801</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D5">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F5" t="b">
         <v>0</v>
@@ -899,13 +878,13 @@
         <v>0.40972222222222199</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C6" t="s">
         <v>26</v>
       </c>
       <c r="D6">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E6" t="s">
         <v>41</v>
@@ -919,16 +898,16 @@
         <v>0.41666666666666702</v>
       </c>
       <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7">
         <v>6</v>
       </c>
-      <c r="C7" t="s">
-        <v>43</v>
-      </c>
-      <c r="D7">
-        <v>8</v>
-      </c>
       <c r="E7" t="s">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="F7" t="b">
         <v>0</v>
@@ -939,16 +918,16 @@
         <v>0.42361111111111099</v>
       </c>
       <c r="B8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="D8">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E8" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="F8" t="b">
         <v>0</v>
@@ -959,16 +938,16 @@
         <v>0.43055555555555602</v>
       </c>
       <c r="B9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="D9">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E9" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="F9" t="b">
         <v>0</v>
@@ -979,16 +958,16 @@
         <v>0.4375</v>
       </c>
       <c r="B10">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D10">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E10" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F10" t="b">
         <v>0</v>
@@ -999,16 +978,16 @@
         <v>0.44444444444444497</v>
       </c>
       <c r="B11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D11">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E11" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F11" t="b">
         <v>0</v>
@@ -1019,13 +998,13 @@
         <v>0.45138888888888901</v>
       </c>
       <c r="B12">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C12" t="s">
         <v>27</v>
       </c>
       <c r="D12">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E12" t="s">
         <v>41</v>
@@ -1039,16 +1018,16 @@
         <v>0.45833333333333398</v>
       </c>
       <c r="B13">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>47</v>
-      </c>
-      <c r="D13">
-        <v>8</v>
+        <v>45</v>
+      </c>
+      <c r="D13" t="s">
+        <v>40</v>
       </c>
       <c r="E13" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="F13" t="b">
         <v>0</v>
@@ -1059,16 +1038,16 @@
         <v>0.46527777777777801</v>
       </c>
       <c r="B14">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D14">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E14" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F14" t="b">
         <v>0</v>
@@ -1079,10 +1058,10 @@
         <v>0.47222222222222299</v>
       </c>
       <c r="B15">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="D15">
         <v>6</v>
@@ -1099,13 +1078,13 @@
         <v>0.47916666666666702</v>
       </c>
       <c r="B16">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C16" t="s">
         <v>31</v>
       </c>
       <c r="D16">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E16" t="s">
         <v>41</v>
@@ -1119,16 +1098,16 @@
         <v>0.48611111111111099</v>
       </c>
       <c r="B17">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C17" t="s">
         <v>31</v>
       </c>
       <c r="D17">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E17" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="F17" t="b">
         <v>1</v>

</xml_diff>